<commit_message>
Ship multi Allowed IP, focus check-in alerts, and Cost Analyzer department filters to live EC2.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/OneView_Table_Structure.xlsx
+++ b/docs/OneView_Table_Structure.xlsx
@@ -690,7 +690,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I110"/>
+  <dimension ref="A1:I111"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3854,13 +3854,66 @@
       </c>
     </row>
     <row r="110">
+      <c r="A110" t="str">
+        <v/>
+      </c>
+      <c r="B110" t="str">
+        <v/>
+      </c>
+      <c r="C110" t="str">
+        <v/>
+      </c>
+      <c r="D110" t="str">
+        <v/>
+      </c>
       <c r="E110" t="str">
         <v>INTEGER</v>
       </c>
+      <c r="F110" t="str">
+        <v/>
+      </c>
+      <c r="G110" t="str">
+        <v/>
+      </c>
+      <c r="H110" t="str">
+        <v/>
+      </c>
+      <c r="I110" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111">
+        <v>1</v>
+      </c>
+      <c r="B111" t="str">
+        <v>employees</v>
+      </c>
+      <c r="C111">
+        <v>16</v>
+      </c>
+      <c r="D111" t="str">
+        <v>allowed_ip</v>
+      </c>
+      <c r="E111" t="str">
+        <v>VARCHAR</v>
+      </c>
+      <c r="F111" t="str">
+        <v>255</v>
+      </c>
+      <c r="G111" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="H111" t="str">
+        <v>Optional login IP restriction. Comma-separated IPv4/IPv6 (max 10). NULL/empty = any IP.</v>
+      </c>
+      <c r="I111" t="str">
+        <v>Optional; Each value valid IP; Login matches any listed IP</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I110"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I111"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3956,7 +4009,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4046,10 +4099,17 @@
         <v>Planner allocations, confirmations, reports snapshots, weekly check-in</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Allowed IP</v>
+      </c>
+      <c r="B12" t="str">
+        <v>employees.allowed_ip: comma-separated IPs; POST /auth/login (and /login/continue) allow when reverse-proxy client IP matches any entry. Empty/NULL = no restriction. IP from connection (req.ip), not body.</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>